<commit_message>
Update sample data and validation rules
</commit_message>
<xml_diff>
--- a/table1_rule.xlsx
+++ b/table1_rule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DICT\Desktop\Divide Rule\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84E207B1-209C-474B-A062-7D41BF8667A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C72BB5D9-F412-4E61-959C-2AABBC382CB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet3" sheetId="4" state="hidden" r:id="rId1"/>
@@ -132,107 +132,6 @@
 Select only from the accepted values. Must be all capital.</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Fixed values only: 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>SOLE PROPRIETORSHIP</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">; </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">
-ONE PERSON CORPORATION</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>;</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">
-PARTNERSHIP</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>;</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">
-CORPORATION</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>;</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve"> or</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">
-COOPERATIVE</t>
-    </r>
-  </si>
-  <si>
     <t>CORPORATION</t>
   </si>
   <si>
@@ -710,6 +609,102 @@
   </si>
   <si>
     <t>Main Office</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Fixed values only: 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t>SOLE PROPRIETORSHIP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">
+ONE PERSON CORPORATION</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t>;</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">
+PARTNERSHIP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t>;</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">
+CORPORATION</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t>;</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve"> or</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">
+COOPERATIVE</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -719,7 +714,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -766,6 +761,12 @@
       <color theme="1"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -799,7 +800,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -837,6 +838,9 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1266,42 +1270,42 @@
       <c r="C5" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="100.5" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="E6" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C7" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>31</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>32</v>
       </c>
       <c r="E7" s="10">
         <v>46107</v>
@@ -1309,53 +1313,53 @@
     </row>
     <row r="8" spans="1:5" ht="130.5" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C8" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="101.25" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C9" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="57" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C10" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="E10" s="5" t="s">
         <v>41</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
@@ -1367,101 +1371,101 @@
     </row>
     <row r="12" spans="1:5" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>43</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>44</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>17</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="57" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B13" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="E13" s="13" t="s">
         <v>48</v>
-      </c>
-      <c r="E13" s="13" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C14" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="E14" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="B15" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="E15" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C16" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B17" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>62</v>
-      </c>
       <c r="D17" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>3</v>
@@ -1469,16 +1473,16 @@
     </row>
     <row r="18" spans="1:5" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A18" s="14" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>4</v>
@@ -1486,135 +1490,135 @@
     </row>
     <row r="19" spans="1:5" ht="43.5" x14ac:dyDescent="0.2">
       <c r="A19" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="B19" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C19" s="5" t="s">
+      <c r="D19" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="E19" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="57" x14ac:dyDescent="0.2">
       <c r="A20" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B20" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C20" s="5" t="s">
+      <c r="D20" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="57" x14ac:dyDescent="0.2">
       <c r="A21" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C21" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="D21" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="E21" s="2" t="s">
         <v>74</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A22" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C22" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="B22" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C22" s="5" t="s">
+      <c r="D22" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E22" s="2" t="s">
         <v>77</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A23" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="B23" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C23" s="5" t="s">
+      <c r="D23" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>80</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A24" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="B24" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C24" s="5" t="s">
+      <c r="D24" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E24" s="2" t="s">
         <v>83</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="57" x14ac:dyDescent="0.2">
       <c r="A25" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C25" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E25" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A26" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="B26" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C26" s="5" t="s">
+      <c r="D26" s="5" t="s">
         <v>89</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>90</v>
       </c>
       <c r="E26" s="2">
         <v>1400101001</v>
@@ -1622,16 +1626,16 @@
     </row>
     <row r="27" spans="1:5" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A27" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="B27" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C27" s="5" t="s">
+      <c r="D27" s="5" t="s">
         <v>92</v>
-      </c>
-      <c r="D27" s="5" t="s">
-        <v>93</v>
       </c>
       <c r="E27" s="2">
         <v>1</v>
@@ -1639,67 +1643,67 @@
     </row>
     <row r="28" spans="1:5" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C28" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="E28" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="D28" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A29" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C29" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="D29" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="D29" s="8" t="s">
+      <c r="E29" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C30" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D30" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="E30" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C31" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D31" s="7" t="s">
         <v>106</v>
-      </c>
-      <c r="D31" s="7" t="s">
-        <v>107</v>
       </c>
       <c r="E31" s="2">
         <v>20000</v>
@@ -1707,16 +1711,16 @@
     </row>
     <row r="32" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C32" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="B32" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C32" s="5" t="s">
+      <c r="D32" s="5" t="s">
         <v>109</v>
-      </c>
-      <c r="D32" s="5" t="s">
-        <v>110</v>
       </c>
       <c r="E32" s="2">
         <v>100</v>
@@ -1724,16 +1728,16 @@
     </row>
     <row r="33" spans="1:5" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C33" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="B33" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C33" s="5" t="s">
+      <c r="D33" s="5" t="s">
         <v>112</v>
-      </c>
-      <c r="D33" s="5" t="s">
-        <v>113</v>
       </c>
       <c r="E33" s="2">
         <v>10</v>
@@ -1741,16 +1745,16 @@
     </row>
     <row r="34" spans="1:5" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C34" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="B34" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>115</v>
-      </c>
       <c r="D34" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E34" s="2">
         <v>5</v>
@@ -1758,16 +1762,16 @@
     </row>
     <row r="35" spans="1:5" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C35" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="B35" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C35" s="5" t="s">
+      <c r="D35" s="5" t="s">
         <v>117</v>
-      </c>
-      <c r="D35" s="5" t="s">
-        <v>118</v>
       </c>
       <c r="E35" s="2">
         <v>8</v>
@@ -1775,16 +1779,16 @@
     </row>
     <row r="36" spans="1:5" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C36" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="B36" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>120</v>
-      </c>
       <c r="D36" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E36" s="2">
         <v>2</v>
@@ -1792,16 +1796,16 @@
     </row>
     <row r="37" spans="1:5" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A37" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C37" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="B37" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C37" s="5" t="s">
-        <v>122</v>
-      </c>
       <c r="D37" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E37" s="2">
         <v>0</v>
@@ -1809,16 +1813,16 @@
     </row>
     <row r="38" spans="1:5" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A38" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C38" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="B38" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C38" s="5" t="s">
-        <v>124</v>
-      </c>
       <c r="D38" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E38" s="2">
         <v>2</v>
@@ -1826,19 +1830,19 @@
     </row>
     <row r="39" spans="1:5" ht="99.75" x14ac:dyDescent="0.2">
       <c r="A39" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C39" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="B39" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C39" s="5" t="s">
+      <c r="D39" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="D39" s="5" t="s">
+      <c r="E39" s="2" t="s">
         <v>127</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>